<commit_message>
fix documentation bug; optics quantities were incorrect (legacy 0.8 m lattice numbers)
</commit_message>
<xml_diff>
--- a/demo_parameters.xlsx
+++ b/demo_parameters.xlsx
@@ -428,7 +428,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27.84"/>
@@ -484,7 +484,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>6</v>
@@ -504,7 +504,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>38.5</v>
+        <v>-61.5</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>6</v>
@@ -524,7 +524,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>20.3</v>
+        <v>-19.7</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>6</v>

</xml_diff>